<commit_message>
Add Kling 2.6 Motion Control page
</commit_message>
<xml_diff>
--- a/docs/model-costs.xlsx
+++ b/docs/model-costs.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="296">
   <si>
     <t>工作表</t>
   </si>
@@ -1271,6 +1271,41 @@
   </si>
   <si>
     <t>KIE模型页 pricingDescCn：720p $0.14/s，1080p $0.24/s。</t>
+  </si>
+  <si>
+    <t>Kling 2.6 Motion Control</t>
+  </si>
+  <si>
+    <t>kling-2-6-motion-control</t>
+  </si>
+  <si>
+    <t>每输出秒:
+KIE独立成本待核实
+Toolaze临时收入 $0.1100 / 输出秒
+Toolaze临时定价 22 积分 / 输出秒
+成本率待确认
+毛利率待确认</t>
+  </si>
+  <si>
+    <t>66+ 积分</t>
+  </si>
+  <si>
+    <t>720p × 3秒（参考视频最短时长）</t>
+  </si>
+  <si>
+    <t>KIE 独立成本待核实</t>
+  </si>
+  <si>
+    <t>KIE 模型页参数已核实; 独立 pricing/registry 成本待核实; functions/_shared/generation-credits.mjs; src/lib/generation-credits.ts</t>
+  </si>
+  <si>
+    <t>https://kie.ai/kling-2.6-motion-control</t>
+  </si>
+  <si>
+    <t>KIE页面参数支持 Image 3-10秒 / Video 3-30秒；当前 Toolaze 暂按 Kling 2.6 标准无音频成本 $0.055/s 映射 22 credits/s，不能视为 Motion Control 独立成本已核实。</t>
+  </si>
+  <si>
+    <t>按上传参考视频的有效时长向上取整后计费；Image 3-10秒，Video 3-30秒</t>
   </si>
 </sst>
 </file>
@@ -2273,7 +2308,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -3158,17 +3193,19 @@
         <v>99</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>230</v>
+        <v>286</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>231</v>
+        <v>287</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
+      <c r="H18" s="2" t="s">
+        <v>288</v>
+      </c>
       <c r="I18" s="2" t="s">
-        <v>232</v>
+        <v>288</v>
       </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
@@ -3176,25 +3213,25 @@
         <v>211</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>233</v>
+        <v>289</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>234</v>
+        <v>290</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>25</v>
+        <v>291</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>26</v>
+        <v>292</v>
       </c>
       <c r="Q18" s="4" t="s">
-        <v>235</v>
+        <v>293</v>
       </c>
       <c r="R18" s="2" t="s">
-        <v>236</v>
+        <v>294</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>117</v>
+        <v>295</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="90" customHeight="1">
@@ -3205,17 +3242,17 @@
         <v>99</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
@@ -3223,7 +3260,7 @@
         <v>211</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="N19" s="2" t="s">
         <v>234</v>
@@ -3235,10 +3272,10 @@
         <v>26</v>
       </c>
       <c r="Q19" s="4" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="R19" s="2" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="S19" s="2" t="s">
         <v>117</v>
@@ -3252,30 +3289,28 @@
         <v>99</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
-      <c r="H20" s="2" t="s">
-        <v>245</v>
-      </c>
+      <c r="H20" s="2"/>
       <c r="I20" s="2" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2" t="s">
-        <v>22</v>
+        <v>211</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>168</v>
+        <v>240</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="O20" s="2" t="s">
         <v>25</v>
@@ -3284,13 +3319,13 @@
         <v>26</v>
       </c>
       <c r="Q20" s="4" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="R20" s="2" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="S20" s="2" t="s">
-        <v>250</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:19" ht="90" customHeight="1">
@@ -3301,19 +3336,19 @@
         <v>99</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
@@ -3321,7 +3356,7 @@
         <v>22</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>255</v>
+        <v>168</v>
       </c>
       <c r="N21" s="2" t="s">
         <v>247</v>
@@ -3336,7 +3371,7 @@
         <v>248</v>
       </c>
       <c r="R21" s="2" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="S21" s="2" t="s">
         <v>250</v>
@@ -3350,19 +3385,19 @@
         <v>99</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
@@ -3370,7 +3405,7 @@
         <v>22</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="N22" s="2" t="s">
         <v>247</v>
@@ -3385,7 +3420,7 @@
         <v>248</v>
       </c>
       <c r="R22" s="2" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="S22" s="2" t="s">
         <v>250</v>
@@ -3399,34 +3434,30 @@
         <v>99</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>265</v>
-      </c>
+        <v>258</v>
+      </c>
+      <c r="E23" s="2"/>
       <c r="F23" s="2"/>
-      <c r="G23" s="2" t="s">
-        <v>266</v>
-      </c>
+      <c r="G23" s="2"/>
       <c r="H23" s="2" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2" t="s">
-        <v>269</v>
+        <v>22</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>271</v>
+        <v>247</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>25</v>
@@ -3435,13 +3466,13 @@
         <v>26</v>
       </c>
       <c r="Q23" s="4" t="s">
-        <v>272</v>
+        <v>248</v>
       </c>
       <c r="R23" s="2" t="s">
-        <v>152</v>
+        <v>262</v>
       </c>
       <c r="S23" s="2" t="s">
-        <v>153</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" spans="1:19" ht="90" customHeight="1">
@@ -3452,30 +3483,34 @@
         <v>99</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>274</v>
-      </c>
-      <c r="E24" s="2"/>
+        <v>264</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>265</v>
+      </c>
       <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
+      <c r="G24" s="2" t="s">
+        <v>266</v>
+      </c>
       <c r="H24" s="2" t="s">
-        <v>210</v>
+        <v>267</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2" t="s">
-        <v>181</v>
+        <v>269</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>221</v>
+        <v>271</v>
       </c>
       <c r="O24" s="2" t="s">
         <v>25</v>
@@ -3484,13 +3519,13 @@
         <v>26</v>
       </c>
       <c r="Q24" s="4" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="R24" s="2" t="s">
-        <v>278</v>
+        <v>152</v>
       </c>
       <c r="S24" s="2" t="s">
-        <v>117</v>
+        <v>153</v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="90" customHeight="1">
@@ -3501,19 +3536,19 @@
         <v>99</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2" t="s">
-        <v>281</v>
+        <v>210</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
@@ -3521,7 +3556,7 @@
         <v>181</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="N25" s="2" t="s">
         <v>221</v>
@@ -3533,17 +3568,66 @@
         <v>26</v>
       </c>
       <c r="Q25" s="4" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="R25" s="2" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="S25" s="2" t="s">
         <v>117</v>
       </c>
     </row>
+    <row r="26" spans="1:19" ht="90" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="M26" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="O26" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q26" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="R26" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="S26" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S25"/>
+  <autoFilter ref="A1:S26"/>
   <hyperlinks>
     <hyperlink ref="Q2" r:id="rId1"/>
     <hyperlink ref="Q3" r:id="rId2"/>
@@ -3561,14 +3645,15 @@
     <hyperlink ref="Q15" r:id="rId14"/>
     <hyperlink ref="Q16" r:id="rId15"/>
     <hyperlink ref="Q17" r:id="rId16"/>
-    <hyperlink ref="Q18" r:id="rId17"/>
-    <hyperlink ref="Q19" r:id="rId18"/>
-    <hyperlink ref="Q20" r:id="rId19"/>
-    <hyperlink ref="Q21" r:id="rId20"/>
-    <hyperlink ref="Q22" r:id="rId21"/>
-    <hyperlink ref="Q23" r:id="rId22"/>
-    <hyperlink ref="Q24" r:id="rId23"/>
-    <hyperlink ref="Q25" r:id="rId24"/>
+    <hyperlink ref="Q18" r:id="rId25"/>
+    <hyperlink ref="Q19" r:id="rId17"/>
+    <hyperlink ref="Q20" r:id="rId18"/>
+    <hyperlink ref="Q21" r:id="rId19"/>
+    <hyperlink ref="Q22" r:id="rId20"/>
+    <hyperlink ref="Q23" r:id="rId21"/>
+    <hyperlink ref="Q24" r:id="rId22"/>
+    <hyperlink ref="Q25" r:id="rId23"/>
+    <hyperlink ref="Q26" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>